<commit_message>
fix(pricing): fix base price fallback, coupon combination logic and candidate discovery for MNL-002309 & PR3-000099
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode_test.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode_test.xlsx
@@ -13,10 +13,10 @@
     <sheet name="Processed_Logs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$C$306</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Failed_Orders'!$A$1:$D$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Completed_Orders'!$A$1:$C$150</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Processed_Logs'!$A$1:$I$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$C$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Failed_Orders'!$A$1:$D$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Completed_Orders'!$A$1:$C$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Processed_Logs'!$A$1:$I$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -319,7 +319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C306"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="4" min="1" max="1"/>
@@ -351,11 +351,7 @@
           <t>SU564M5AA</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>SU564M5AA</t>
-        </is>
-      </c>
+      <c r="C2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr"/>
@@ -364,11 +360,7 @@
           <t>SU564M5PC</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>SU564M5PC</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
@@ -377,11 +369,7 @@
           <t>SU564M9WN</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>SU564M9WN</t>
-        </is>
-      </c>
+      <c r="C4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr"/>
@@ -390,11 +378,7 @@
           <t>SU564M9B0</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>SU564M9B0</t>
-        </is>
-      </c>
+      <c r="C5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr"/>
@@ -403,11 +387,7 @@
           <t>SU564MB82</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>SU564MB82</t>
-        </is>
-      </c>
+      <c r="C6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr"/>
@@ -416,11 +396,7 @@
           <t>SU564MANM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>SU564MANM</t>
-        </is>
-      </c>
+      <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr"/>
@@ -429,11 +405,7 @@
           <t>SU564M928</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>SU564M928</t>
-        </is>
-      </c>
+      <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr"/>
@@ -1540,11 +1512,7 @@
       <c r="C208" s="3" t="inlineStr"/>
     </row>
     <row r="209">
-      <c r="A209" s="3" t="inlineStr">
-        <is>
-          <t>2610205CASVS3V</t>
-        </is>
-      </c>
+      <c r="A209" s="3" t="inlineStr"/>
       <c r="B209" s="3" t="inlineStr"/>
       <c r="C209" s="3" t="inlineStr"/>
     </row>
@@ -1584,159 +1552,119 @@
       <c r="C216" s="3" t="inlineStr"/>
     </row>
     <row r="217">
-      <c r="A217" s="3" t="inlineStr">
-        <is>
-          <t>2610205CBKM7J1</t>
-        </is>
-      </c>
+      <c r="A217" s="3" t="inlineStr"/>
       <c r="B217" s="3" t="inlineStr"/>
       <c r="C217" s="3" t="inlineStr"/>
     </row>
     <row r="218">
-      <c r="A218" s="3" t="inlineStr">
-        <is>
-          <t>2610205CDYVPEK</t>
-        </is>
-      </c>
+      <c r="A218" s="3" t="inlineStr"/>
       <c r="B218" s="3" t="inlineStr"/>
       <c r="C218" s="3" t="inlineStr"/>
     </row>
     <row r="219">
-      <c r="A219" s="3" t="inlineStr">
-        <is>
-          <t>2610205CT8S089</t>
-        </is>
-      </c>
+      <c r="A219" s="3" t="inlineStr"/>
       <c r="B219" s="3" t="inlineStr"/>
       <c r="C219" s="3" t="inlineStr"/>
     </row>
     <row r="220">
-      <c r="A220" s="3" t="inlineStr">
-        <is>
-          <t>2610205D58Q0TW</t>
-        </is>
-      </c>
+      <c r="A220" s="3" t="inlineStr"/>
       <c r="B220" s="3" t="inlineStr"/>
       <c r="C220" s="3" t="inlineStr"/>
     </row>
     <row r="221">
-      <c r="A221" s="3" t="inlineStr">
-        <is>
-          <t>2610205DHCUBGF</t>
-        </is>
-      </c>
+      <c r="A221" s="3" t="inlineStr"/>
       <c r="B221" s="3" t="inlineStr"/>
       <c r="C221" s="3" t="inlineStr"/>
     </row>
     <row r="222">
-      <c r="A222" s="3" t="inlineStr">
-        <is>
-          <t>2610205FNF148X</t>
-        </is>
-      </c>
+      <c r="A222" s="3" t="inlineStr"/>
       <c r="B222" s="3" t="inlineStr"/>
       <c r="C222" s="3" t="inlineStr"/>
     </row>
     <row r="223">
-      <c r="A223" s="3" t="inlineStr">
-        <is>
-          <t>2610205FQKPQXJ</t>
-        </is>
-      </c>
+      <c r="A223" s="3" t="inlineStr"/>
       <c r="B223" s="3" t="inlineStr"/>
       <c r="C223" s="3" t="inlineStr"/>
     </row>
     <row r="224">
-      <c r="A224" s="3" t="inlineStr">
-        <is>
-          <t>2610205G2A487N</t>
-        </is>
-      </c>
+      <c r="A224" s="3" t="inlineStr"/>
       <c r="B224" s="3" t="inlineStr"/>
       <c r="C224" s="3" t="inlineStr"/>
     </row>
     <row r="225">
-      <c r="A225" s="3" t="inlineStr">
-        <is>
-          <t>2610205G9TDVEK</t>
-        </is>
-      </c>
+      <c r="A225" s="3" t="inlineStr"/>
       <c r="B225" s="3" t="inlineStr"/>
       <c r="C225" s="3" t="inlineStr"/>
     </row>
     <row r="226">
-      <c r="A226" s="3" t="inlineStr">
-        <is>
-          <t>2610205GG0RJP3</t>
-        </is>
-      </c>
+      <c r="A226" s="3" t="inlineStr"/>
       <c r="B226" s="3" t="inlineStr"/>
       <c r="C226" s="3" t="inlineStr"/>
     </row>
     <row r="227">
-      <c r="A227" s="3" t="inlineStr">
-        <is>
-          <t>2610205GTHDX0T</t>
-        </is>
-      </c>
+      <c r="A227" s="3" t="inlineStr"/>
       <c r="B227" s="3" t="inlineStr"/>
       <c r="C227" s="3" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="3" t="inlineStr">
-        <is>
-          <t>2610205JC2CXHC</t>
-        </is>
-      </c>
+      <c r="A228" s="3" t="inlineStr"/>
       <c r="B228" s="3" t="inlineStr"/>
       <c r="C228" s="3" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
         <is>
-          <t>2610205K0V2QCE</t>
+          <t>2610218A2WCX78</t>
         </is>
       </c>
       <c r="B229" s="3" t="inlineStr"/>
       <c r="C229" s="3" t="inlineStr"/>
     </row>
     <row r="230">
-      <c r="A230" s="3" t="inlineStr">
-        <is>
-          <t>2610205K1KX372</t>
-        </is>
-      </c>
+      <c r="A230" s="3" t="inlineStr"/>
       <c r="B230" s="3" t="inlineStr"/>
       <c r="C230" s="3" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
         <is>
-          <t>2610205KU39SPS</t>
+          <t>2610218AQHBP4W</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr"/>
       <c r="C231" s="3" t="inlineStr"/>
     </row>
     <row r="232">
-      <c r="A232" s="3" t="inlineStr"/>
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>2610218AVNB1FC</t>
+        </is>
+      </c>
       <c r="B232" s="3" t="inlineStr"/>
       <c r="C232" s="3" t="inlineStr"/>
     </row>
     <row r="233">
-      <c r="A233" s="3" t="inlineStr"/>
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>2610218B0GCAQ7</t>
+        </is>
+      </c>
       <c r="B233" s="3" t="inlineStr"/>
       <c r="C233" s="3" t="inlineStr"/>
     </row>
     <row r="234">
-      <c r="A234" s="3" t="inlineStr"/>
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>2610218B5CQQXM</t>
+        </is>
+      </c>
       <c r="B234" s="3" t="inlineStr"/>
       <c r="C234" s="3" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
         <is>
-          <t>2610205KXHY6J1</t>
+          <t>2610218B7GGDFK</t>
         </is>
       </c>
       <c r="B235" s="3" t="inlineStr"/>
@@ -1745,7 +1673,7 @@
     <row r="236">
       <c r="A236" s="3" t="inlineStr">
         <is>
-          <t>2610205MG0TMXX</t>
+          <t>2610218BA3FF4J</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr"/>
@@ -1754,7 +1682,7 @@
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
         <is>
-          <t>2610205MSWCKV5</t>
+          <t>2610218BCU6S4C</t>
         </is>
       </c>
       <c r="B237" s="3" t="inlineStr"/>
@@ -1763,7 +1691,7 @@
     <row r="238">
       <c r="A238" s="3" t="inlineStr">
         <is>
-          <t>2610205P8RJJAR</t>
+          <t>2610218DKJ9V5R</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr"/>
@@ -1772,7 +1700,7 @@
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
         <is>
-          <t>2610205PB5T1B5</t>
+          <t>2610218E7H6T2H</t>
         </is>
       </c>
       <c r="B239" s="3" t="inlineStr"/>
@@ -1781,7 +1709,7 @@
     <row r="240">
       <c r="A240" s="3" t="inlineStr">
         <is>
-          <t>2610205PWM4F63</t>
+          <t>2610218ESUQDK6</t>
         </is>
       </c>
       <c r="B240" s="3" t="inlineStr"/>
@@ -1790,7 +1718,7 @@
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
         <is>
-          <t>2610205QF228C5</t>
+          <t>2610218EYY7KAX</t>
         </is>
       </c>
       <c r="B241" s="3" t="inlineStr"/>
@@ -1799,7 +1727,7 @@
     <row r="242">
       <c r="A242" s="3" t="inlineStr">
         <is>
-          <t>2610205REK3DPP</t>
+          <t>2610218F8UENKE</t>
         </is>
       </c>
       <c r="B242" s="3" t="inlineStr"/>
@@ -1808,7 +1736,7 @@
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
         <is>
-          <t>2610205RGG3S2U</t>
+          <t>2610218G11UDDF</t>
         </is>
       </c>
       <c r="B243" s="3" t="inlineStr"/>
@@ -1817,7 +1745,7 @@
     <row r="244">
       <c r="A244" s="3" t="inlineStr">
         <is>
-          <t>2610205RH6YHMS</t>
+          <t>2610218G4FEJWN</t>
         </is>
       </c>
       <c r="B244" s="3" t="inlineStr"/>
@@ -1826,7 +1754,7 @@
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
         <is>
-          <t>2610205S3DPYRR</t>
+          <t>2610218G8BDVQW</t>
         </is>
       </c>
       <c r="B245" s="3" t="inlineStr"/>
@@ -1835,7 +1763,7 @@
     <row r="246">
       <c r="A246" s="3" t="inlineStr">
         <is>
-          <t>2610205TF1TFHF</t>
+          <t>2610218GBQ6XRH</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr"/>
@@ -1844,7 +1772,7 @@
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
         <is>
-          <t>2610205TS55GMF</t>
+          <t>2610218GP5YVPD</t>
         </is>
       </c>
       <c r="B247" s="3" t="inlineStr"/>
@@ -1853,7 +1781,7 @@
     <row r="248">
       <c r="A248" s="3" t="inlineStr">
         <is>
-          <t>2610205U0DUH9Q</t>
+          <t>2610218GY18E99</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr"/>
@@ -1862,7 +1790,7 @@
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
         <is>
-          <t>2610205U47X2N9</t>
+          <t>2610218J886G5W</t>
         </is>
       </c>
       <c r="B249" s="3" t="inlineStr"/>
@@ -1871,25 +1799,21 @@
     <row r="250">
       <c r="A250" s="3" t="inlineStr">
         <is>
-          <t>2610205U7TABYF</t>
+          <t>2610218JCCPEF3</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr"/>
       <c r="C250" s="3" t="inlineStr"/>
     </row>
     <row r="251">
-      <c r="A251" s="3" t="inlineStr">
-        <is>
-          <t>2610205VC5TDB3</t>
-        </is>
-      </c>
+      <c r="A251" s="3" t="inlineStr"/>
       <c r="B251" s="3" t="inlineStr"/>
       <c r="C251" s="3" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="inlineStr">
         <is>
-          <t>2610205VD4AG0N</t>
+          <t>2610218MXF2W3H</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr"/>
@@ -1898,7 +1822,7 @@
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
         <is>
-          <t>2610205VQ8JQ47</t>
+          <t>2610228RM3AEUH</t>
         </is>
       </c>
       <c r="B253" s="3" t="inlineStr"/>
@@ -1907,7 +1831,7 @@
     <row r="254">
       <c r="A254" s="3" t="inlineStr">
         <is>
-          <t>2610205VY0GVA1</t>
+          <t>2610228RQMQNX5</t>
         </is>
       </c>
       <c r="B254" s="3" t="inlineStr"/>
@@ -1916,7 +1840,7 @@
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
         <is>
-          <t>2610205W9H7S74</t>
+          <t>2610228S1BMCY3</t>
         </is>
       </c>
       <c r="B255" s="3" t="inlineStr"/>
@@ -1925,7 +1849,7 @@
     <row r="256">
       <c r="A256" s="3" t="inlineStr">
         <is>
-          <t>2610205XC6AHM4</t>
+          <t>2610228S6A0634</t>
         </is>
       </c>
       <c r="B256" s="3" t="inlineStr"/>
@@ -1934,7 +1858,7 @@
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
         <is>
-          <t>2610205YRQ3T98</t>
+          <t>2610228TCJF8TJ</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr"/>
@@ -1943,7 +1867,7 @@
     <row r="258">
       <c r="A258" s="3" t="inlineStr">
         <is>
-          <t>26102061CEQGXC</t>
+          <t>2610228TJXKXDG</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr"/>
@@ -1952,7 +1876,7 @@
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
         <is>
-          <t>261020629NB0D3</t>
+          <t>2610228TM5QH3H</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr"/>
@@ -1961,7 +1885,7 @@
     <row r="260">
       <c r="A260" s="3" t="inlineStr">
         <is>
-          <t>26102062QA3DQK</t>
+          <t>2610228TPF30GW</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr"/>
@@ -1970,7 +1894,7 @@
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
         <is>
-          <t>26102063D18SXA</t>
+          <t>2610228U3A4JWC</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr"/>
@@ -1979,21 +1903,25 @@
     <row r="262">
       <c r="A262" s="3" t="inlineStr">
         <is>
-          <t>26102064M0QFCW</t>
+          <t>2610228U5V70DP</t>
         </is>
       </c>
       <c r="B262" s="3" t="inlineStr"/>
       <c r="C262" s="3" t="inlineStr"/>
     </row>
     <row r="263">
-      <c r="A263" s="3" t="inlineStr"/>
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>2610228UVQMWDA</t>
+        </is>
+      </c>
       <c r="B263" s="3" t="inlineStr"/>
       <c r="C263" s="3" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="inlineStr">
         <is>
-          <t>26102164T38JEK</t>
+          <t>2610228WVXTXFH</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr"/>
@@ -2002,7 +1930,7 @@
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
         <is>
-          <t>26102167KCF00F</t>
+          <t>2610228WY6BNJ0</t>
         </is>
       </c>
       <c r="B265" s="3" t="inlineStr"/>
@@ -2011,7 +1939,7 @@
     <row r="266">
       <c r="A266" s="3" t="inlineStr">
         <is>
-          <t>26102167WX2F3M</t>
+          <t>2610228XKY1A2F</t>
         </is>
       </c>
       <c r="B266" s="3" t="inlineStr"/>
@@ -2020,7 +1948,7 @@
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
         <is>
-          <t>261021698D3D7C</t>
+          <t>261022933MPUE1</t>
         </is>
       </c>
       <c r="B267" s="3" t="inlineStr"/>
@@ -2029,7 +1957,7 @@
     <row r="268">
       <c r="A268" s="3" t="inlineStr">
         <is>
-          <t>261021699RWGC3</t>
+          <t>26102298JPKH12</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr"/>
@@ -2038,7 +1966,7 @@
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
         <is>
-          <t>2610216AQB3V23</t>
+          <t>261022991HH9F2</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr"/>
@@ -2047,7 +1975,7 @@
     <row r="270">
       <c r="A270" s="3" t="inlineStr">
         <is>
-          <t>2610216AXF06QF</t>
+          <t>2610229BYS1YCY</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr"/>
@@ -2056,7 +1984,7 @@
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
         <is>
-          <t>2610216AXSJ055</t>
+          <t>2610229DK1AT9G</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr"/>
@@ -2065,7 +1993,7 @@
     <row r="272">
       <c r="A272" s="3" t="inlineStr">
         <is>
-          <t>2610216BF435GM</t>
+          <t>2610229DQ412YT</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr"/>
@@ -2074,7 +2002,7 @@
     <row r="273">
       <c r="A273" s="3" t="inlineStr">
         <is>
-          <t>2610216BV8Q9F0</t>
+          <t>2610229EGS5FMY</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr"/>
@@ -2083,7 +2011,7 @@
     <row r="274">
       <c r="A274" s="3" t="inlineStr">
         <is>
-          <t>2610216CUF74MR</t>
+          <t>2610229GUVC4XF</t>
         </is>
       </c>
       <c r="B274" s="3" t="inlineStr"/>
@@ -2092,7 +2020,7 @@
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
         <is>
-          <t>2610216DBN2PX2</t>
+          <t>2610229J3QE34G</t>
         </is>
       </c>
       <c r="B275" s="3" t="inlineStr"/>
@@ -2101,7 +2029,7 @@
     <row r="276">
       <c r="A276" s="3" t="inlineStr">
         <is>
-          <t>2610216J6FD2VU</t>
+          <t>2610229JNGS9N4</t>
         </is>
       </c>
       <c r="B276" s="3" t="inlineStr"/>
@@ -2110,7 +2038,7 @@
     <row r="277">
       <c r="A277" s="3" t="inlineStr">
         <is>
-          <t>2610216JQRGAP6</t>
+          <t>2610229M4PDMS6</t>
         </is>
       </c>
       <c r="B277" s="3" t="inlineStr"/>
@@ -2119,7 +2047,7 @@
     <row r="278">
       <c r="A278" s="3" t="inlineStr">
         <is>
-          <t>2610216MAU45XE</t>
+          <t>2610229MG8F05S</t>
         </is>
       </c>
       <c r="B278" s="3" t="inlineStr"/>
@@ -2128,7 +2056,7 @@
     <row r="279">
       <c r="A279" s="3" t="inlineStr">
         <is>
-          <t>2610216SNPJAQA</t>
+          <t>2610229MHFJ44T</t>
         </is>
       </c>
       <c r="B279" s="3" t="inlineStr"/>
@@ -2137,7 +2065,7 @@
     <row r="280">
       <c r="A280" s="3" t="inlineStr">
         <is>
-          <t>2610216UJC80PE</t>
+          <t>2610229P3U8XPD</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr"/>
@@ -2146,7 +2074,7 @@
     <row r="281">
       <c r="A281" s="3" t="inlineStr">
         <is>
-          <t>2610216W9YSWT0</t>
+          <t>2610229Q0RC40D</t>
         </is>
       </c>
       <c r="B281" s="3" t="inlineStr"/>
@@ -2155,7 +2083,7 @@
     <row r="282">
       <c r="A282" s="3" t="inlineStr">
         <is>
-          <t>2610216YFS8D82</t>
+          <t>2610229Q17JXN0</t>
         </is>
       </c>
       <c r="B282" s="3" t="inlineStr"/>
@@ -2164,7 +2092,7 @@
     <row r="283">
       <c r="A283" s="3" t="inlineStr">
         <is>
-          <t>26102171E1FDBJ</t>
+          <t>2610229QQVCTYY</t>
         </is>
       </c>
       <c r="B283" s="3" t="inlineStr"/>
@@ -2173,7 +2101,7 @@
     <row r="284">
       <c r="A284" s="3" t="inlineStr">
         <is>
-          <t>26102172AJ41BU</t>
+          <t>2610229R9F3D3X</t>
         </is>
       </c>
       <c r="B284" s="3" t="inlineStr"/>
@@ -2182,7 +2110,7 @@
     <row r="285">
       <c r="A285" s="3" t="inlineStr">
         <is>
-          <t>26102173QYJSBU</t>
+          <t>2610229RQ6PKUG</t>
         </is>
       </c>
       <c r="B285" s="3" t="inlineStr"/>
@@ -2191,7 +2119,7 @@
     <row r="286">
       <c r="A286" s="3" t="inlineStr">
         <is>
-          <t>26102174G7TQWP</t>
+          <t>2610229RTMBCB4</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr"/>
@@ -2200,7 +2128,7 @@
     <row r="287">
       <c r="A287" s="3" t="inlineStr">
         <is>
-          <t>26102174V4CWWB</t>
+          <t>2610229SA847C1</t>
         </is>
       </c>
       <c r="B287" s="3" t="inlineStr"/>
@@ -2209,7 +2137,7 @@
     <row r="288">
       <c r="A288" s="3" t="inlineStr">
         <is>
-          <t>2610217620F70U</t>
+          <t>2610229SG5VYRN</t>
         </is>
       </c>
       <c r="B288" s="3" t="inlineStr"/>
@@ -2218,167 +2146,14 @@
     <row r="289">
       <c r="A289" s="3" t="inlineStr">
         <is>
-          <t>26102176SGXHMV</t>
+          <t>2610229SS8SW92</t>
         </is>
       </c>
       <c r="B289" s="3" t="inlineStr"/>
       <c r="C289" s="3" t="inlineStr"/>
     </row>
-    <row r="290">
-      <c r="A290" s="3" t="inlineStr">
-        <is>
-          <t>26102177UH3KJG</t>
-        </is>
-      </c>
-      <c r="B290" s="3" t="inlineStr"/>
-      <c r="C290" s="3" t="inlineStr"/>
-    </row>
-    <row r="291">
-      <c r="A291" s="3" t="inlineStr">
-        <is>
-          <t>26102178RKWC4W</t>
-        </is>
-      </c>
-      <c r="B291" s="3" t="inlineStr"/>
-      <c r="C291" s="3" t="inlineStr"/>
-    </row>
-    <row r="292">
-      <c r="A292" s="3" t="inlineStr">
-        <is>
-          <t>26102178VHRNC6</t>
-        </is>
-      </c>
-      <c r="B292" s="3" t="inlineStr"/>
-      <c r="C292" s="3" t="inlineStr"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="3" t="inlineStr">
-        <is>
-          <t>261021790BUYXV</t>
-        </is>
-      </c>
-      <c r="B293" s="3" t="inlineStr"/>
-      <c r="C293" s="3" t="inlineStr"/>
-    </row>
-    <row r="294">
-      <c r="A294" s="3" t="inlineStr">
-        <is>
-          <t>261021796URVP2</t>
-        </is>
-      </c>
-      <c r="B294" s="3" t="inlineStr"/>
-      <c r="C294" s="3" t="inlineStr"/>
-    </row>
-    <row r="295">
-      <c r="A295" s="3" t="inlineStr">
-        <is>
-          <t>26102179FRWGJ1</t>
-        </is>
-      </c>
-      <c r="B295" s="3" t="inlineStr"/>
-      <c r="C295" s="3" t="inlineStr"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="3" t="inlineStr">
-        <is>
-          <t>26102179Q69ND5</t>
-        </is>
-      </c>
-      <c r="B296" s="3" t="inlineStr"/>
-      <c r="C296" s="3" t="inlineStr"/>
-    </row>
-    <row r="297">
-      <c r="A297" s="3" t="inlineStr">
-        <is>
-          <t>2610217A4NBTHV</t>
-        </is>
-      </c>
-      <c r="B297" s="3" t="inlineStr"/>
-      <c r="C297" s="3" t="inlineStr"/>
-    </row>
-    <row r="298">
-      <c r="A298" s="3" t="inlineStr">
-        <is>
-          <t>2610217BJ7JR54</t>
-        </is>
-      </c>
-      <c r="B298" s="3" t="inlineStr"/>
-      <c r="C298" s="3" t="inlineStr"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="3" t="inlineStr">
-        <is>
-          <t>2610217C726Y1D</t>
-        </is>
-      </c>
-      <c r="B299" s="3" t="inlineStr"/>
-      <c r="C299" s="3" t="inlineStr"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="3" t="inlineStr">
-        <is>
-          <t>2610217C7P5S3N</t>
-        </is>
-      </c>
-      <c r="B300" s="3" t="inlineStr"/>
-      <c r="C300" s="3" t="inlineStr"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="3" t="inlineStr">
-        <is>
-          <t>2610217CFUH5DX</t>
-        </is>
-      </c>
-      <c r="B301" s="3" t="inlineStr"/>
-      <c r="C301" s="3" t="inlineStr"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="3" t="inlineStr">
-        <is>
-          <t>2610217CNGQPQY</t>
-        </is>
-      </c>
-      <c r="B302" s="3" t="inlineStr"/>
-      <c r="C302" s="3" t="inlineStr"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="3" t="inlineStr">
-        <is>
-          <t>2610217CSP7HYN</t>
-        </is>
-      </c>
-      <c r="B303" s="3" t="inlineStr"/>
-      <c r="C303" s="3" t="inlineStr"/>
-    </row>
-    <row r="304">
-      <c r="A304" s="3" t="inlineStr">
-        <is>
-          <t>2610217E9PKXCW</t>
-        </is>
-      </c>
-      <c r="B304" s="3" t="inlineStr"/>
-      <c r="C304" s="3" t="inlineStr"/>
-    </row>
-    <row r="305">
-      <c r="A305" s="3" t="inlineStr">
-        <is>
-          <t>2610217ETN7KWS</t>
-        </is>
-      </c>
-      <c r="B305" s="3" t="inlineStr"/>
-      <c r="C305" s="3" t="inlineStr"/>
-    </row>
-    <row r="306">
-      <c r="A306" s="3" t="inlineStr">
-        <is>
-          <t>2610217F7GA8NP</t>
-        </is>
-      </c>
-      <c r="B306" s="3" t="inlineStr"/>
-      <c r="C306" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C306"/>
+  <autoFilter ref="A1:C289"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2389,7 +2164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="4" min="1" max="1"/>
@@ -3335,8 +3110,66 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:28:27</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>261021882U112W</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: COA-002069 (วันที่: 2026-10-21 19:06, ราคาที่ต้องออกบิล: 0.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-21 19:06
+COA-002069 [ไม่จำหน่าย] MSI Folding Wagon รถเข็น ของแถมสำหรับจอ MSI ที่ร่วมรายการเท่านั้น
+ยิงขายขึ้น 3,000.00 บาท
+ลูกค้าซื้อราคา 0.00 บาท
+ขอวิธีปรับราคาครับ
+💡 [ระบบคำนวณแนะนำ] พบคูปองบน SMCO ที่ลดแล้วได้ราคา 0.00 บาท พอดีเป๊ะ:
+   • แนะนำ: 'DC2607230007' (ส่วนลด 3,000.00 บาท)
+   • บันทึกใส่คอลัมน์ 'suggested_cp' ใน cp_data.xlsx เรียบร้อยแล้ว (เปิดตรวจสอบและคัดลอกได้)
+ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:29:23</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>261021885HSPGR</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: MNL-002577 (วันที่: 2026-10-21 19:07, ราคาที่ต้องออกบิล: 9051.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-21 19:07
+MNL-002577 MSI Gaming Monitor MAG 321UPD E14 - 31.5"/IPS/4K 144Hz,FHD 288Hz/1ms/AMD FreeSync Premium/3Y*3 MNL-002577
+ยิงขายขึ้น 9,571.00 บาท
+ลูกค้าซื้อราคา 9,051.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D33"/>
+  <autoFilter ref="A1:D35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3347,7 +3180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C150"/>
+  <dimension ref="A1:C152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="4" min="1" max="1"/>
@@ -5905,8 +5738,42 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:30:15</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>2610218863WM9A</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ราคาตรงตั้งแต่แรก/All OK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:31:16</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>2610218A1EN9RQ</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C150"/>
+  <autoFilter ref="A1:C152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5917,7 +5784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="4" min="1" max="1"/>
@@ -5978,7 +5845,7 @@
         </is>
       </c>
     </row>
-    <row r="2" s="4">
+    <row r="2" hidden="1" s="4">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:35:53</t>
@@ -6017,7 +5884,7 @@
         </is>
       </c>
     </row>
-    <row r="3" s="4">
+    <row r="3" hidden="1" s="4">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:36:48</t>
@@ -6056,7 +5923,7 @@
         </is>
       </c>
     </row>
-    <row r="4" s="4">
+    <row r="4" hidden="1" s="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:37:31</t>
@@ -6095,7 +5962,7 @@
         </is>
       </c>
     </row>
-    <row r="5" s="4">
+    <row r="5" hidden="1" s="4">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:37:54</t>
@@ -6134,7 +6001,7 @@
         </is>
       </c>
     </row>
-    <row r="6" s="4">
+    <row r="6" hidden="1" s="4">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:19</t>
@@ -6173,7 +6040,7 @@
         </is>
       </c>
     </row>
-    <row r="7" s="4">
+    <row r="7" hidden="1" s="4">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:19</t>
@@ -6212,7 +6079,7 @@
         </is>
       </c>
     </row>
-    <row r="8" s="4">
+    <row r="8" hidden="1" s="4">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:19</t>
@@ -6251,7 +6118,7 @@
         </is>
       </c>
     </row>
-    <row r="9" s="4">
+    <row r="9" hidden="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:19</t>
@@ -6290,7 +6157,7 @@
         </is>
       </c>
     </row>
-    <row r="10" s="4">
+    <row r="10" hidden="1" s="4">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:44</t>
@@ -6329,7 +6196,7 @@
         </is>
       </c>
     </row>
-    <row r="11" s="4">
+    <row r="11" hidden="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:38:44</t>
@@ -6368,7 +6235,7 @@
         </is>
       </c>
     </row>
-    <row r="12" s="4">
+    <row r="12" hidden="1" s="4">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:39:07</t>
@@ -6407,7 +6274,7 @@
         </is>
       </c>
     </row>
-    <row r="13" s="4">
+    <row r="13" hidden="1" s="4">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:39:52</t>
@@ -6446,7 +6313,7 @@
         </is>
       </c>
     </row>
-    <row r="14" s="4">
+    <row r="14" hidden="1" s="4">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:40:21</t>
@@ -6485,7 +6352,7 @@
         </is>
       </c>
     </row>
-    <row r="15" s="4">
+    <row r="15" hidden="1" s="4">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:41:03</t>
@@ -6524,7 +6391,7 @@
         </is>
       </c>
     </row>
-    <row r="16" s="4">
+    <row r="16" hidden="1" s="4">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:41:28</t>
@@ -6563,7 +6430,7 @@
         </is>
       </c>
     </row>
-    <row r="17" s="4">
+    <row r="17" hidden="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:42:27</t>
@@ -6603,7 +6470,7 @@
         </is>
       </c>
     </row>
-    <row r="18" s="4">
+    <row r="18" hidden="1" s="4">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:42:51</t>
@@ -6642,7 +6509,7 @@
         </is>
       </c>
     </row>
-    <row r="19" s="4">
+    <row r="19" hidden="1" s="4">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:43:33</t>
@@ -6681,7 +6548,7 @@
         </is>
       </c>
     </row>
-    <row r="20" s="4">
+    <row r="20" hidden="1" s="4">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:44:12</t>
@@ -6720,7 +6587,7 @@
         </is>
       </c>
     </row>
-    <row r="21" s="4">
+    <row r="21" hidden="1" s="4">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:45:02</t>
@@ -6759,7 +6626,7 @@
         </is>
       </c>
     </row>
-    <row r="22" s="4">
+    <row r="22" hidden="1" s="4">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:45:25</t>
@@ -6798,7 +6665,7 @@
         </is>
       </c>
     </row>
-    <row r="23" s="4">
+    <row r="23" hidden="1" s="4">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:45:48</t>
@@ -6837,7 +6704,7 @@
         </is>
       </c>
     </row>
-    <row r="24" s="4">
+    <row r="24" hidden="1" s="4">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:46:32</t>
@@ -6876,7 +6743,7 @@
         </is>
       </c>
     </row>
-    <row r="25" s="4">
+    <row r="25" hidden="1" s="4">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:46:32</t>
@@ -6915,7 +6782,7 @@
         </is>
       </c>
     </row>
-    <row r="26" s="4">
+    <row r="26" hidden="1" s="4">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:46:32</t>
@@ -6954,7 +6821,7 @@
         </is>
       </c>
     </row>
-    <row r="27" s="4">
+    <row r="27" hidden="1" s="4">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:46:32</t>
@@ -6993,7 +6860,7 @@
         </is>
       </c>
     </row>
-    <row r="28" s="4">
+    <row r="28" hidden="1" s="4">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:46:32</t>
@@ -7032,7 +6899,7 @@
         </is>
       </c>
     </row>
-    <row r="29" s="4">
+    <row r="29" hidden="1" s="4">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:47:06</t>
@@ -7072,7 +6939,7 @@
         </is>
       </c>
     </row>
-    <row r="30" s="4">
+    <row r="30" hidden="1" s="4">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:47:46</t>
@@ -7111,7 +6978,7 @@
         </is>
       </c>
     </row>
-    <row r="31" s="4">
+    <row r="31" hidden="1" s="4">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:48:23</t>
@@ -7150,7 +7017,7 @@
         </is>
       </c>
     </row>
-    <row r="32" s="4">
+    <row r="32" hidden="1" s="4">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:49:04</t>
@@ -7189,7 +7056,7 @@
         </is>
       </c>
     </row>
-    <row r="33" s="4">
+    <row r="33" hidden="1" s="4">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:49:31</t>
@@ -7228,7 +7095,7 @@
         </is>
       </c>
     </row>
-    <row r="34" s="4">
+    <row r="34" hidden="1" s="4">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:49:56</t>
@@ -7267,7 +7134,7 @@
         </is>
       </c>
     </row>
-    <row r="35" s="4">
+    <row r="35" hidden="1" s="4">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:50:31</t>
@@ -7313,7 +7180,7 @@
         </is>
       </c>
     </row>
-    <row r="36" s="4">
+    <row r="36" hidden="1" s="4">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:51:00</t>
@@ -7352,7 +7219,7 @@
         </is>
       </c>
     </row>
-    <row r="37" s="4">
+    <row r="37" hidden="1" s="4">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:51:42</t>
@@ -7392,7 +7259,7 @@
         </is>
       </c>
     </row>
-    <row r="38" s="4">
+    <row r="38" hidden="1" s="4">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:52:05</t>
@@ -7431,7 +7298,7 @@
         </is>
       </c>
     </row>
-    <row r="39" s="4">
+    <row r="39" hidden="1" s="4">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:52:05</t>
@@ -7470,7 +7337,7 @@
         </is>
       </c>
     </row>
-    <row r="40" s="4">
+    <row r="40" hidden="1" s="4">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:52:45</t>
@@ -7509,7 +7376,7 @@
         </is>
       </c>
     </row>
-    <row r="41" s="4">
+    <row r="41" hidden="1" s="4">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:53:40</t>
@@ -7548,7 +7415,7 @@
         </is>
       </c>
     </row>
-    <row r="42" s="4">
+    <row r="42" hidden="1" s="4">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:53:40</t>
@@ -7587,7 +7454,7 @@
         </is>
       </c>
     </row>
-    <row r="43" s="4">
+    <row r="43" hidden="1" s="4">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:53:40</t>
@@ -7626,7 +7493,7 @@
         </is>
       </c>
     </row>
-    <row r="44" s="4">
+    <row r="44" hidden="1" s="4">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:54:06</t>
@@ -7665,7 +7532,7 @@
         </is>
       </c>
     </row>
-    <row r="45" s="4">
+    <row r="45" hidden="1" s="4">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:54:59</t>
@@ -7704,7 +7571,7 @@
         </is>
       </c>
     </row>
-    <row r="46" s="4">
+    <row r="46" hidden="1" s="4">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:55:56</t>
@@ -7743,7 +7610,7 @@
         </is>
       </c>
     </row>
-    <row r="47" s="4">
+    <row r="47" hidden="1" s="4">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:56:36</t>
@@ -7782,7 +7649,7 @@
         </is>
       </c>
     </row>
-    <row r="48" s="4">
+    <row r="48" hidden="1" s="4">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:57:40</t>
@@ -7821,7 +7688,7 @@
         </is>
       </c>
     </row>
-    <row r="49" s="4">
+    <row r="49" hidden="1" s="4">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:58:04</t>
@@ -7860,7 +7727,7 @@
         </is>
       </c>
     </row>
-    <row r="50" s="4">
+    <row r="50" hidden="1" s="4">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:58:49</t>
@@ -7899,7 +7766,7 @@
         </is>
       </c>
     </row>
-    <row r="51" s="4">
+    <row r="51" hidden="1" s="4">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 15:59:27</t>
@@ -7938,7 +7805,7 @@
         </is>
       </c>
     </row>
-    <row r="52" s="4">
+    <row r="52" hidden="1" s="4">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:00:08</t>
@@ -7977,7 +7844,7 @@
         </is>
       </c>
     </row>
-    <row r="53" s="4">
+    <row r="53" hidden="1" s="4">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:00:53</t>
@@ -8016,7 +7883,7 @@
         </is>
       </c>
     </row>
-    <row r="54" s="4">
+    <row r="54" hidden="1" s="4">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:00:53</t>
@@ -8055,7 +7922,7 @@
         </is>
       </c>
     </row>
-    <row r="55" s="4">
+    <row r="55" hidden="1" s="4">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:01:23</t>
@@ -8094,7 +7961,7 @@
         </is>
       </c>
     </row>
-    <row r="56" s="4">
+    <row r="56" hidden="1" s="4">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:02:16</t>
@@ -8133,7 +8000,7 @@
         </is>
       </c>
     </row>
-    <row r="57" s="4">
+    <row r="57" hidden="1" s="4">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:02:58</t>
@@ -8172,7 +8039,7 @@
         </is>
       </c>
     </row>
-    <row r="58" s="4">
+    <row r="58" hidden="1" s="4">
       <c r="A58" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:03:47</t>
@@ -8211,7 +8078,7 @@
         </is>
       </c>
     </row>
-    <row r="59" s="4">
+    <row r="59" hidden="1" s="4">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:04:22</t>
@@ -8250,7 +8117,7 @@
         </is>
       </c>
     </row>
-    <row r="60" s="4">
+    <row r="60" hidden="1" s="4">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:05:08</t>
@@ -8289,7 +8156,7 @@
         </is>
       </c>
     </row>
-    <row r="61" s="4">
+    <row r="61" hidden="1" s="4">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:06:03</t>
@@ -8329,7 +8196,7 @@
         </is>
       </c>
     </row>
-    <row r="62" s="4">
+    <row r="62" hidden="1" s="4">
       <c r="A62" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:06:42</t>
@@ -8368,7 +8235,7 @@
         </is>
       </c>
     </row>
-    <row r="63" s="4">
+    <row r="63" hidden="1" s="4">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:08:02</t>
@@ -8408,7 +8275,7 @@
         </is>
       </c>
     </row>
-    <row r="64" s="4">
+    <row r="64" hidden="1" s="4">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:08:47</t>
@@ -8447,7 +8314,7 @@
         </is>
       </c>
     </row>
-    <row r="65" s="4">
+    <row r="65" hidden="1" s="4">
       <c r="A65" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:09:12</t>
@@ -8486,7 +8353,7 @@
         </is>
       </c>
     </row>
-    <row r="66" s="4">
+    <row r="66" hidden="1" s="4">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:09:58</t>
@@ -8525,7 +8392,7 @@
         </is>
       </c>
     </row>
-    <row r="67" s="4">
+    <row r="67" hidden="1" s="4">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:11:03</t>
@@ -8565,7 +8432,7 @@
         </is>
       </c>
     </row>
-    <row r="68" s="4">
+    <row r="68" hidden="1" s="4">
       <c r="A68" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:11:31</t>
@@ -8604,7 +8471,7 @@
         </is>
       </c>
     </row>
-    <row r="69" s="4">
+    <row r="69" hidden="1" s="4">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:11:55</t>
@@ -8643,7 +8510,7 @@
         </is>
       </c>
     </row>
-    <row r="70" s="4">
+    <row r="70" hidden="1" s="4">
       <c r="A70" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:12:23</t>
@@ -8682,7 +8549,7 @@
         </is>
       </c>
     </row>
-    <row r="71" s="4">
+    <row r="71" hidden="1" s="4">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:13:16</t>
@@ -8721,7 +8588,7 @@
         </is>
       </c>
     </row>
-    <row r="72" s="4">
+    <row r="72" hidden="1" s="4">
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:14:05</t>
@@ -8760,7 +8627,7 @@
         </is>
       </c>
     </row>
-    <row r="73" s="4">
+    <row r="73" hidden="1" s="4">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:14:44</t>
@@ -8799,7 +8666,7 @@
         </is>
       </c>
     </row>
-    <row r="74" s="4">
+    <row r="74" hidden="1" s="4">
       <c r="A74" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:15:22</t>
@@ -8843,7 +8710,7 @@
         </is>
       </c>
     </row>
-    <row r="75" s="4">
+    <row r="75" hidden="1" s="4">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:16:10</t>
@@ -8882,7 +8749,7 @@
         </is>
       </c>
     </row>
-    <row r="76" s="4">
+    <row r="76" hidden="1" s="4">
       <c r="A76" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:16:53</t>
@@ -8921,7 +8788,7 @@
         </is>
       </c>
     </row>
-    <row r="77" s="4">
+    <row r="77" hidden="1" s="4">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:17:38</t>
@@ -8960,7 +8827,7 @@
         </is>
       </c>
     </row>
-    <row r="78" s="4">
+    <row r="78" hidden="1" s="4">
       <c r="A78" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:18:23</t>
@@ -8999,7 +8866,7 @@
         </is>
       </c>
     </row>
-    <row r="79" s="4">
+    <row r="79" hidden="1" s="4">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:19:13</t>
@@ -9038,7 +8905,7 @@
         </is>
       </c>
     </row>
-    <row r="80" s="4">
+    <row r="80" hidden="1" s="4">
       <c r="A80" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:19:13</t>
@@ -9077,7 +8944,7 @@
         </is>
       </c>
     </row>
-    <row r="81" s="4">
+    <row r="81" hidden="1" s="4">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:19:13</t>
@@ -9116,7 +8983,7 @@
         </is>
       </c>
     </row>
-    <row r="82" s="4">
+    <row r="82" hidden="1" s="4">
       <c r="A82" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:20:02</t>
@@ -9155,7 +9022,7 @@
         </is>
       </c>
     </row>
-    <row r="83" s="4">
+    <row r="83" hidden="1" s="4">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:20:49</t>
@@ -9199,7 +9066,7 @@
         </is>
       </c>
     </row>
-    <row r="84" s="4">
+    <row r="84" hidden="1" s="4">
       <c r="A84" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:21:50</t>
@@ -9239,7 +9106,7 @@
         </is>
       </c>
     </row>
-    <row r="85" s="4">
+    <row r="85" hidden="1" s="4">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:22:35</t>
@@ -9278,7 +9145,7 @@
         </is>
       </c>
     </row>
-    <row r="86" s="4">
+    <row r="86" hidden="1" s="4">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:23:06</t>
@@ -9322,7 +9189,7 @@
         </is>
       </c>
     </row>
-    <row r="87" s="4">
+    <row r="87" hidden="1" s="4">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:23:49</t>
@@ -9361,7 +9228,7 @@
         </is>
       </c>
     </row>
-    <row r="88" s="4">
+    <row r="88" hidden="1" s="4">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:24:28</t>
@@ -9405,7 +9272,7 @@
         </is>
       </c>
     </row>
-    <row r="89" s="4">
+    <row r="89" hidden="1" s="4">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:25:35</t>
@@ -9444,7 +9311,7 @@
         </is>
       </c>
     </row>
-    <row r="90" s="4">
+    <row r="90" hidden="1" s="4">
       <c r="A90" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:25:59</t>
@@ -9483,7 +9350,7 @@
         </is>
       </c>
     </row>
-    <row r="91" s="4">
+    <row r="91" hidden="1" s="4">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:26:38</t>
@@ -9522,7 +9389,7 @@
         </is>
       </c>
     </row>
-    <row r="92" s="4">
+    <row r="92" hidden="1" s="4">
       <c r="A92" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:27:18</t>
@@ -9561,7 +9428,7 @@
         </is>
       </c>
     </row>
-    <row r="93" s="4">
+    <row r="93" hidden="1" s="4">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:27:57</t>
@@ -9600,7 +9467,7 @@
         </is>
       </c>
     </row>
-    <row r="94" s="4">
+    <row r="94" hidden="1" s="4">
       <c r="A94" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:28:41</t>
@@ -9639,7 +9506,7 @@
         </is>
       </c>
     </row>
-    <row r="95" s="4">
+    <row r="95" hidden="1" s="4">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:29:25</t>
@@ -9678,7 +9545,7 @@
         </is>
       </c>
     </row>
-    <row r="96" s="4">
+    <row r="96" hidden="1" s="4">
       <c r="A96" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:30:08</t>
@@ -9717,7 +9584,7 @@
         </is>
       </c>
     </row>
-    <row r="97" s="4">
+    <row r="97" hidden="1" s="4">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:30:29</t>
@@ -9756,7 +9623,7 @@
         </is>
       </c>
     </row>
-    <row r="98" s="4">
+    <row r="98" hidden="1" s="4">
       <c r="A98" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:31:21</t>
@@ -9795,7 +9662,7 @@
         </is>
       </c>
     </row>
-    <row r="99" s="4">
+    <row r="99" hidden="1" s="4">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:32:04</t>
@@ -9834,7 +9701,7 @@
         </is>
       </c>
     </row>
-    <row r="100" s="4">
+    <row r="100" hidden="1" s="4">
       <c r="A100" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:32:39</t>
@@ -9874,7 +9741,7 @@
         </is>
       </c>
     </row>
-    <row r="101" s="4">
+    <row r="101" hidden="1" s="4">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:33:34</t>
@@ -9914,7 +9781,7 @@
         </is>
       </c>
     </row>
-    <row r="102" s="4">
+    <row r="102" hidden="1" s="4">
       <c r="A102" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:34:14</t>
@@ -9953,7 +9820,7 @@
         </is>
       </c>
     </row>
-    <row r="103" s="4">
+    <row r="103" hidden="1" s="4">
       <c r="A103" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:35:26</t>
@@ -9992,7 +9859,7 @@
         </is>
       </c>
     </row>
-    <row r="104" s="4">
+    <row r="104" hidden="1" s="4">
       <c r="A104" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:35:26</t>
@@ -10031,7 +9898,7 @@
         </is>
       </c>
     </row>
-    <row r="105" s="4">
+    <row r="105" hidden="1" s="4">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:35:26</t>
@@ -10070,7 +9937,7 @@
         </is>
       </c>
     </row>
-    <row r="106" s="4">
+    <row r="106" hidden="1" s="4">
       <c r="A106" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:35:54</t>
@@ -10109,7 +9976,7 @@
         </is>
       </c>
     </row>
-    <row r="107" s="4">
+    <row r="107" hidden="1" s="4">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:35:54</t>
@@ -10148,7 +10015,7 @@
         </is>
       </c>
     </row>
-    <row r="108" s="4">
+    <row r="108" hidden="1" s="4">
       <c r="A108" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:36:36</t>
@@ -10187,7 +10054,7 @@
         </is>
       </c>
     </row>
-    <row r="109" s="4">
+    <row r="109" hidden="1" s="4">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:37:15</t>
@@ -10226,7 +10093,7 @@
         </is>
       </c>
     </row>
-    <row r="110" s="4">
+    <row r="110" hidden="1" s="4">
       <c r="A110" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:37:38</t>
@@ -10265,7 +10132,7 @@
         </is>
       </c>
     </row>
-    <row r="111" s="4">
+    <row r="111" hidden="1" s="4">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:38:00</t>
@@ -10304,7 +10171,7 @@
         </is>
       </c>
     </row>
-    <row r="112" s="4">
+    <row r="112" hidden="1" s="4">
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:39:44</t>
@@ -10344,7 +10211,7 @@
         </is>
       </c>
     </row>
-    <row r="113" s="4">
+    <row r="113" hidden="1" s="4">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:40:23</t>
@@ -10384,7 +10251,7 @@
         </is>
       </c>
     </row>
-    <row r="114" s="4">
+    <row r="114" hidden="1" s="4">
       <c r="A114" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:40:46</t>
@@ -10423,7 +10290,7 @@
         </is>
       </c>
     </row>
-    <row r="115" s="4">
+    <row r="115" hidden="1" s="4">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:41:11</t>
@@ -10462,7 +10329,7 @@
         </is>
       </c>
     </row>
-    <row r="116" s="4">
+    <row r="116" hidden="1" s="4">
       <c r="A116" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:41:54</t>
@@ -10501,7 +10368,7 @@
         </is>
       </c>
     </row>
-    <row r="117" s="4">
+    <row r="117" hidden="1" s="4">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:42:21</t>
@@ -10540,7 +10407,7 @@
         </is>
       </c>
     </row>
-    <row r="118" s="4">
+    <row r="118" hidden="1" s="4">
       <c r="A118" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:42:41</t>
@@ -10579,7 +10446,7 @@
         </is>
       </c>
     </row>
-    <row r="119" s="4">
+    <row r="119" hidden="1" s="4">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:42:47</t>
@@ -10606,7 +10473,7 @@
       <c r="H119" s="3" t="inlineStr"/>
       <c r="I119" s="3" t="inlineStr"/>
     </row>
-    <row r="120" s="4">
+    <row r="120" hidden="1" s="4">
       <c r="A120" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:43:27</t>
@@ -10645,7 +10512,7 @@
         </is>
       </c>
     </row>
-    <row r="121" s="4">
+    <row r="121" hidden="1" s="4">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:44:08</t>
@@ -10684,7 +10551,7 @@
         </is>
       </c>
     </row>
-    <row r="122" s="4">
+    <row r="122" hidden="1" s="4">
       <c r="A122" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:44:47</t>
@@ -10724,7 +10591,7 @@
         </is>
       </c>
     </row>
-    <row r="123" s="4">
+    <row r="123" hidden="1" s="4">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:45:25</t>
@@ -10764,7 +10631,7 @@
         </is>
       </c>
     </row>
-    <row r="124" s="4">
+    <row r="124" hidden="1" s="4">
       <c r="A124" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:46:05</t>
@@ -10804,7 +10671,7 @@
         </is>
       </c>
     </row>
-    <row r="125" s="4">
+    <row r="125" hidden="1" s="4">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:46:43</t>
@@ -10844,7 +10711,7 @@
         </is>
       </c>
     </row>
-    <row r="126" s="4">
+    <row r="126" hidden="1" s="4">
       <c r="A126" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:47:07</t>
@@ -10883,7 +10750,7 @@
         </is>
       </c>
     </row>
-    <row r="127" s="4">
+    <row r="127" hidden="1" s="4">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:47:46</t>
@@ -10922,7 +10789,7 @@
         </is>
       </c>
     </row>
-    <row r="128" s="4">
+    <row r="128" hidden="1" s="4">
       <c r="A128" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:48:28</t>
@@ -10961,7 +10828,7 @@
         </is>
       </c>
     </row>
-    <row r="129" s="4">
+    <row r="129" hidden="1" s="4">
       <c r="A129" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:49:07</t>
@@ -11000,7 +10867,7 @@
         </is>
       </c>
     </row>
-    <row r="130" s="4">
+    <row r="130" hidden="1" s="4">
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:49:50</t>
@@ -11039,7 +10906,7 @@
         </is>
       </c>
     </row>
-    <row r="131" s="4">
+    <row r="131" hidden="1" s="4">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:50:15</t>
@@ -11078,7 +10945,7 @@
         </is>
       </c>
     </row>
-    <row r="132" s="4">
+    <row r="132" hidden="1" s="4">
       <c r="A132" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:50:39</t>
@@ -11117,7 +10984,7 @@
         </is>
       </c>
     </row>
-    <row r="133" s="4">
+    <row r="133" hidden="1" s="4">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:51:21</t>
@@ -11156,7 +11023,7 @@
         </is>
       </c>
     </row>
-    <row r="134" s="4">
+    <row r="134" hidden="1" s="4">
       <c r="A134" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:51:27</t>
@@ -11183,7 +11050,7 @@
       <c r="H134" s="3" t="inlineStr"/>
       <c r="I134" s="3" t="inlineStr"/>
     </row>
-    <row r="135" s="4">
+    <row r="135" hidden="1" s="4">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:51:27</t>
@@ -11210,7 +11077,7 @@
       <c r="H135" s="3" t="inlineStr"/>
       <c r="I135" s="3" t="inlineStr"/>
     </row>
-    <row r="136" s="4">
+    <row r="136" hidden="1" s="4">
       <c r="A136" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:51:50</t>
@@ -11249,7 +11116,7 @@
         </is>
       </c>
     </row>
-    <row r="137" s="4">
+    <row r="137" hidden="1" s="4">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:52:09</t>
@@ -11288,7 +11155,7 @@
         </is>
       </c>
     </row>
-    <row r="138" s="4">
+    <row r="138" hidden="1" s="4">
       <c r="A138" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:52:46</t>
@@ -11327,7 +11194,7 @@
         </is>
       </c>
     </row>
-    <row r="139" s="4">
+    <row r="139" hidden="1" s="4">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:53:31</t>
@@ -11366,7 +11233,7 @@
         </is>
       </c>
     </row>
-    <row r="140" s="4">
+    <row r="140" hidden="1" s="4">
       <c r="A140" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:54:13</t>
@@ -11405,7 +11272,7 @@
         </is>
       </c>
     </row>
-    <row r="141" s="4">
+    <row r="141" hidden="1" s="4">
       <c r="A141" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:54:52</t>
@@ -11444,7 +11311,7 @@
         </is>
       </c>
     </row>
-    <row r="142" s="4">
+    <row r="142" hidden="1" s="4">
       <c r="A142" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:55:20</t>
@@ -11483,7 +11350,7 @@
         </is>
       </c>
     </row>
-    <row r="143" s="4">
+    <row r="143" hidden="1" s="4">
       <c r="A143" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:56:00</t>
@@ -11522,7 +11389,7 @@
         </is>
       </c>
     </row>
-    <row r="144" s="4">
+    <row r="144" hidden="1" s="4">
       <c r="A144" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:56:23</t>
@@ -11561,7 +11428,7 @@
         </is>
       </c>
     </row>
-    <row r="145" s="4">
+    <row r="145" hidden="1" s="4">
       <c r="A145" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:56:29</t>
@@ -11588,7 +11455,7 @@
       <c r="H145" s="3" t="inlineStr"/>
       <c r="I145" s="3" t="inlineStr"/>
     </row>
-    <row r="146" s="4">
+    <row r="146" hidden="1" s="4">
       <c r="A146" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:56:29</t>
@@ -11615,7 +11482,7 @@
       <c r="H146" s="3" t="inlineStr"/>
       <c r="I146" s="3" t="inlineStr"/>
     </row>
-    <row r="147" s="4">
+    <row r="147" hidden="1" s="4">
       <c r="A147" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:56:29</t>
@@ -11642,7 +11509,7 @@
       <c r="H147" s="3" t="inlineStr"/>
       <c r="I147" s="3" t="inlineStr"/>
     </row>
-    <row r="148" s="4">
+    <row r="148" hidden="1" s="4">
       <c r="A148" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:57:03</t>
@@ -11686,7 +11553,7 @@
         </is>
       </c>
     </row>
-    <row r="149" s="4">
+    <row r="149" hidden="1" s="4">
       <c r="A149" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:57:43</t>
@@ -11725,7 +11592,7 @@
         </is>
       </c>
     </row>
-    <row r="150" s="4">
+    <row r="150" hidden="1" s="4">
       <c r="A150" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:58:23</t>
@@ -11764,7 +11631,7 @@
         </is>
       </c>
     </row>
-    <row r="151" s="4">
+    <row r="151" hidden="1" s="4">
       <c r="A151" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:58:28</t>
@@ -11791,7 +11658,7 @@
       <c r="H151" s="3" t="inlineStr"/>
       <c r="I151" s="3" t="inlineStr"/>
     </row>
-    <row r="152" s="4">
+    <row r="152" hidden="1" s="4">
       <c r="A152" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:58:28</t>
@@ -11818,7 +11685,7 @@
       <c r="H152" s="3" t="inlineStr"/>
       <c r="I152" s="3" t="inlineStr"/>
     </row>
-    <row r="153" s="4">
+    <row r="153" hidden="1" s="4">
       <c r="A153" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:58:28</t>
@@ -11845,7 +11712,7 @@
       <c r="H153" s="3" t="inlineStr"/>
       <c r="I153" s="3" t="inlineStr"/>
     </row>
-    <row r="154" s="4">
+    <row r="154" hidden="1" s="4">
       <c r="A154" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:58:50</t>
@@ -11884,7 +11751,7 @@
         </is>
       </c>
     </row>
-    <row r="155" s="4">
+    <row r="155" hidden="1" s="4">
       <c r="A155" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:59:09</t>
@@ -11923,7 +11790,7 @@
         </is>
       </c>
     </row>
-    <row r="156" s="4">
+    <row r="156" hidden="1" s="4">
       <c r="A156" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 16:59:49</t>
@@ -11962,7 +11829,7 @@
         </is>
       </c>
     </row>
-    <row r="157" s="4">
+    <row r="157" hidden="1" s="4">
       <c r="A157" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:00:29</t>
@@ -12001,7 +11868,7 @@
         </is>
       </c>
     </row>
-    <row r="158" s="4">
+    <row r="158" hidden="1" s="4">
       <c r="A158" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:01:08</t>
@@ -12040,7 +11907,7 @@
         </is>
       </c>
     </row>
-    <row r="159" s="4">
+    <row r="159" hidden="1" s="4">
       <c r="A159" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:01:42</t>
@@ -12080,7 +11947,7 @@
         </is>
       </c>
     </row>
-    <row r="160" s="4">
+    <row r="160" hidden="1" s="4">
       <c r="A160" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:02:02</t>
@@ -12119,7 +11986,7 @@
         </is>
       </c>
     </row>
-    <row r="161" s="4">
+    <row r="161" hidden="1" s="4">
       <c r="A161" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:02:53</t>
@@ -12158,7 +12025,7 @@
         </is>
       </c>
     </row>
-    <row r="162" s="4">
+    <row r="162" hidden="1" s="4">
       <c r="A162" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:03:32</t>
@@ -12198,7 +12065,7 @@
         </is>
       </c>
     </row>
-    <row r="163" s="4">
+    <row r="163" hidden="1" s="4">
       <c r="A163" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:03:56</t>
@@ -12237,7 +12104,7 @@
         </is>
       </c>
     </row>
-    <row r="164" s="4">
+    <row r="164" hidden="1" s="4">
       <c r="A164" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:04:39</t>
@@ -12276,7 +12143,7 @@
         </is>
       </c>
     </row>
-    <row r="165" s="4">
+    <row r="165" hidden="1" s="4">
       <c r="A165" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:04:39</t>
@@ -12315,7 +12182,7 @@
         </is>
       </c>
     </row>
-    <row r="166" s="4">
+    <row r="166" hidden="1" s="4">
       <c r="A166" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:05:04</t>
@@ -12354,7 +12221,7 @@
         </is>
       </c>
     </row>
-    <row r="167" s="4">
+    <row r="167" hidden="1" s="4">
       <c r="A167" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:05:44</t>
@@ -12393,7 +12260,7 @@
         </is>
       </c>
     </row>
-    <row r="168" s="4">
+    <row r="168" hidden="1" s="4">
       <c r="A168" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:05:44</t>
@@ -12432,7 +12299,7 @@
         </is>
       </c>
     </row>
-    <row r="169" s="4">
+    <row r="169" hidden="1" s="4">
       <c r="A169" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:05:44</t>
@@ -12471,7 +12338,7 @@
         </is>
       </c>
     </row>
-    <row r="170" s="4">
+    <row r="170" hidden="1" s="4">
       <c r="A170" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:05:44</t>
@@ -12510,7 +12377,7 @@
         </is>
       </c>
     </row>
-    <row r="171" s="4">
+    <row r="171" hidden="1" s="4">
       <c r="A171" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:06:04</t>
@@ -12549,7 +12416,7 @@
         </is>
       </c>
     </row>
-    <row r="172" s="4">
+    <row r="172" hidden="1" s="4">
       <c r="A172" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:06:43</t>
@@ -12588,7 +12455,7 @@
         </is>
       </c>
     </row>
-    <row r="173" s="4">
+    <row r="173" hidden="1" s="4">
       <c r="A173" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:07:22</t>
@@ -12627,7 +12494,7 @@
         </is>
       </c>
     </row>
-    <row r="174" s="4">
+    <row r="174" hidden="1" s="4">
       <c r="A174" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:08:00</t>
@@ -12666,7 +12533,7 @@
         </is>
       </c>
     </row>
-    <row r="175" s="4">
+    <row r="175" hidden="1" s="4">
       <c r="A175" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:08:24</t>
@@ -12705,7 +12572,7 @@
         </is>
       </c>
     </row>
-    <row r="176" s="4">
+    <row r="176" hidden="1" s="4">
       <c r="A176" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:09:06</t>
@@ -12744,7 +12611,7 @@
         </is>
       </c>
     </row>
-    <row r="177" s="4">
+    <row r="177" hidden="1" s="4">
       <c r="A177" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:09:49</t>
@@ -12783,7 +12650,7 @@
         </is>
       </c>
     </row>
-    <row r="178" s="4">
+    <row r="178" hidden="1" s="4">
       <c r="A178" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:10:16</t>
@@ -12822,7 +12689,7 @@
         </is>
       </c>
     </row>
-    <row r="179" s="4">
+    <row r="179" hidden="1" s="4">
       <c r="A179" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:10:56</t>
@@ -12861,7 +12728,7 @@
         </is>
       </c>
     </row>
-    <row r="180" s="4">
+    <row r="180" hidden="1" s="4">
       <c r="A180" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:11:21</t>
@@ -12900,7 +12767,7 @@
         </is>
       </c>
     </row>
-    <row r="181" s="4">
+    <row r="181" hidden="1" s="4">
       <c r="A181" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:11:58</t>
@@ -12939,7 +12806,7 @@
         </is>
       </c>
     </row>
-    <row r="182" s="4">
+    <row r="182" hidden="1" s="4">
       <c r="A182" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:12:35</t>
@@ -12979,7 +12846,7 @@
         </is>
       </c>
     </row>
-    <row r="183" s="4">
+    <row r="183" hidden="1" s="4">
       <c r="A183" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:13:00</t>
@@ -13018,7 +12885,7 @@
         </is>
       </c>
     </row>
-    <row r="184" s="4">
+    <row r="184" hidden="1" s="4">
       <c r="A184" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:13:38</t>
@@ -13057,7 +12924,7 @@
         </is>
       </c>
     </row>
-    <row r="185" s="4">
+    <row r="185" hidden="1" s="4">
       <c r="A185" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:14:09</t>
@@ -13103,7 +12970,7 @@
         </is>
       </c>
     </row>
-    <row r="186" s="4">
+    <row r="186" hidden="1" s="4">
       <c r="A186" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:14:49</t>
@@ -13142,7 +13009,7 @@
         </is>
       </c>
     </row>
-    <row r="187" s="4">
+    <row r="187" hidden="1" s="4">
       <c r="A187" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:14:49</t>
@@ -13181,7 +13048,7 @@
         </is>
       </c>
     </row>
-    <row r="188" s="4">
+    <row r="188" hidden="1" s="4">
       <c r="A188" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:15:29</t>
@@ -13220,7 +13087,7 @@
         </is>
       </c>
     </row>
-    <row r="189" s="4">
+    <row r="189" hidden="1" s="4">
       <c r="A189" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:16:07</t>
@@ -13259,7 +13126,7 @@
         </is>
       </c>
     </row>
-    <row r="190" s="4">
+    <row r="190" hidden="1" s="4">
       <c r="A190" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:16:48</t>
@@ -13298,7 +13165,7 @@
         </is>
       </c>
     </row>
-    <row r="191" s="4">
+    <row r="191" hidden="1" s="4">
       <c r="A191" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:17:24</t>
@@ -13337,7 +13204,7 @@
         </is>
       </c>
     </row>
-    <row r="192" s="4">
+    <row r="192" hidden="1" s="4">
       <c r="A192" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:17:45</t>
@@ -13376,7 +13243,7 @@
         </is>
       </c>
     </row>
-    <row r="193" s="4">
+    <row r="193" hidden="1" s="4">
       <c r="A193" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:18:56</t>
@@ -13415,7 +13282,7 @@
         </is>
       </c>
     </row>
-    <row r="194" s="4">
+    <row r="194" hidden="1" s="4">
       <c r="A194" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:18:56</t>
@@ -13454,7 +13321,7 @@
         </is>
       </c>
     </row>
-    <row r="195" s="4">
+    <row r="195" hidden="1" s="4">
       <c r="A195" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:19:38</t>
@@ -13493,7 +13360,7 @@
         </is>
       </c>
     </row>
-    <row r="196" s="4">
+    <row r="196" hidden="1" s="4">
       <c r="A196" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:20:20</t>
@@ -13532,7 +13399,7 @@
         </is>
       </c>
     </row>
-    <row r="197" s="4">
+    <row r="197" hidden="1" s="4">
       <c r="A197" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:21:03</t>
@@ -13571,7 +13438,7 @@
         </is>
       </c>
     </row>
-    <row r="198" s="4">
+    <row r="198" hidden="1" s="4">
       <c r="A198" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:21:26</t>
@@ -13610,7 +13477,7 @@
         </is>
       </c>
     </row>
-    <row r="199" s="4">
+    <row r="199" hidden="1" s="4">
       <c r="A199" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:22:03</t>
@@ -13650,7 +13517,7 @@
         </is>
       </c>
     </row>
-    <row r="200" s="4">
+    <row r="200" hidden="1" s="4">
       <c r="A200" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:22:56</t>
@@ -13689,7 +13556,7 @@
         </is>
       </c>
     </row>
-    <row r="201" s="4">
+    <row r="201" hidden="1" s="4">
       <c r="A201" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:23:40</t>
@@ -13728,7 +13595,7 @@
         </is>
       </c>
     </row>
-    <row r="202" s="4">
+    <row r="202" hidden="1" s="4">
       <c r="A202" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:24:13</t>
@@ -13768,7 +13635,7 @@
         </is>
       </c>
     </row>
-    <row r="203" s="4">
+    <row r="203" hidden="1" s="4">
       <c r="A203" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:24:35</t>
@@ -13807,7 +13674,7 @@
         </is>
       </c>
     </row>
-    <row r="204" s="4">
+    <row r="204" hidden="1" s="4">
       <c r="A204" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:24:35</t>
@@ -13846,7 +13713,7 @@
         </is>
       </c>
     </row>
-    <row r="205" s="4">
+    <row r="205" hidden="1" s="4">
       <c r="A205" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:25:20</t>
@@ -13892,7 +13759,7 @@
         </is>
       </c>
     </row>
-    <row r="206" s="4">
+    <row r="206" hidden="1" s="4">
       <c r="A206" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:26:00</t>
@@ -13932,7 +13799,7 @@
         </is>
       </c>
     </row>
-    <row r="207" s="4">
+    <row r="207" hidden="1" s="4">
       <c r="A207" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:26:48</t>
@@ -13971,7 +13838,7 @@
         </is>
       </c>
     </row>
-    <row r="208" s="4">
+    <row r="208" hidden="1" s="4">
       <c r="A208" s="3" t="inlineStr">
         <is>
           <t>2026-10-21 17:26:48</t>
@@ -14010,8 +13877,174 @@
         </is>
       </c>
     </row>
+    <row r="209" s="4">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:28:26</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>TH260125064166C</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>261021882U112W</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr"/>
+      <c r="E209" s="3" t="inlineStr"/>
+      <c r="F209" s="3" t="inlineStr"/>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: COA-002069 (วันที่: 2026-10-21 19:06, ราคาที่ต้องออกบิล: 0.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-21 19:06
+COA-002069 [ไม่จำหน่าย] MSI Folding Wagon รถเข็น ของแถมสำหรับจอ MSI ที่ร่วมรายการเท่านั้น
+ยิงขายขึ้น 3,000.00 บาท
+ลูกค้าซื้อราคา 0.00 บาท
+ขอวิธีปรับราคาครับ
+💡 [ระบบคำนวณแนะนำ] พบคูปองบน SMCO ที่ลดแล้วได้ราคา 0.00 บาท พอดีเป๊ะ:
+   • แนะนำ: 'DC2607230007' (ส่วนลด 3,000.00 บาท)
+   • บันทึกใส่คอลัมน์ 'suggested_cp' ใน cp_data.xlsx เรียบร้อยแล้ว (เปิดตรวจสอบและคัดลอกได้)
+ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" s="4">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:29:23</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>TH2668202761008</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>261021885HSPGR</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr"/>
+      <c r="E210" s="3" t="inlineStr"/>
+      <c r="F210" s="3" t="inlineStr"/>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: MNL-002577 (วันที่: 2026-10-21 19:07, ราคาที่ต้องออกบิล: 9051.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-21 19:07
+MNL-002577 MSI Gaming Monitor MAG 321UPD E14 - 31.5"/IPS/4K 144Hz,FHD 288Hz/1ms/AMD FreeSync Premium/3Y*3 MNL-002577
+ยิงขายขึ้น 9,571.00 บาท
+ลูกค้าซื้อราคา 9,051.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" s="4">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:30:15</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>TH2615658578600</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>2610218863WM9A</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>2538.0</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>SU564M928</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ราคาตรงตั้งแต่แรก/All OK)</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr"/>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>MNL-002276: POS=2,538.00/เป้า=2,538.00 [ตรง ✅] | Total: POS=2,538.00/เป้า=2,538.00 [ตรง ✅]</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" s="4">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:31:16</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>TH268721603901A</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>2610218A1EN9RQ</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>2781.0</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr"/>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr"/>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>MNL-002412: POS=2,781.00/เป้า=2,781.00 [ตรง ✅] | Total: POS=2,781.00/เป้า=2,781.00 [ตรง ✅]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I208"/>
+  <autoFilter ref="A1:I212"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>